<commit_message>
Story 24.4 review round 1: XLSX fixture with exactness column, LibreOffice check, review order
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014HARNkCaZGyxKh3tp4iZEj
</commit_message>
<xml_diff>
--- a/zobba/fixtures/exports/working-paper.xlsx
+++ b/zobba/fixtures/exports/working-paper.xlsx
@@ -514,7 +514,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exact count</t>
+          <t xml:space="preserve">Count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Count is</t>
         </is>
       </c>
     </row>
@@ -544,6 +549,11 @@
       <c r="C3">
         <v>20</v>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -559,6 +569,11 @@
       <c r="C4">
         <v>960</v>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -574,6 +589,11 @@
       <c r="C5">
         <v>20</v>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -588,6 +608,11 @@
       </c>
       <c r="C6">
         <v>200</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -605,6 +630,11 @@
         <f>SUM(C3:C6)</f>
         <v>1200</v>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>